<commit_message>
Registra encadenes de cuerda y test de sensor pendiente
</commit_message>
<xml_diff>
--- a/escalada/moonboard_entrenamientos.xlsx
+++ b/escalada/moonboard_entrenamientos.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sesiones MoonBoard" sheetId="1" r:id="Rd09b0bfe38ae4dfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sesiones MoonBoard" sheetId="1" r:id="R539f280df7354f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuerda y sensor" sheetId="2" r:id="R0a7f6f0e316c4656"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +21,7 @@
     <x:numFmt numFmtId="203" formatCode="0.00"/>
     <x:numFmt numFmtId="204" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="14">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -70,8 +71,37 @@
       <x:sz val="11"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF243746"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FF243746"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF566B7B"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FF243746"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -86,6 +116,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF3F8"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -121,7 +161,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="41">
+  <x:cellXfs count="57">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -207,6 +247,52 @@
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -819,7 +905,243 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R729e0eb839e1435d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70b3b0de441e4259"/>
   </x:tableParts>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF1F4E78"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="19" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="59" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="42"/>
+      <x:c r="B1" s="42"/>
+      <x:c r="C1" s="42"/>
+      <x:c r="D1" s="42"/>
+      <x:c r="E1" s="42"/>
+      <x:c r="F1" s="42"/>
+      <x:c r="G1" s="42"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="43" t="str">
+        <x:v>Ascensiones de cuerda</x:v>
+      </x:c>
+      <x:c r="B2" s="42"/>
+      <x:c r="C2" s="42"/>
+      <x:c r="D2" s="42"/>
+      <x:c r="E2" s="42"/>
+      <x:c r="F2" s="42"/>
+      <x:c r="G2" s="42"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="42"/>
+      <x:c r="B3" s="42"/>
+      <x:c r="C3" s="42"/>
+      <x:c r="D3" s="42"/>
+      <x:c r="E3" s="42"/>
+      <x:c r="F3" s="42"/>
+      <x:c r="G3" s="42"/>
+    </x:row>
+    <x:row r="4" ht="27" customHeight="1">
+      <x:c r="A4" s="46" t="str">
+        <x:v>Fecha</x:v>
+      </x:c>
+      <x:c r="B4" s="46" t="str">
+        <x:v>Vía</x:v>
+      </x:c>
+      <x:c r="C4" s="46" t="str">
+        <x:v>Zona</x:v>
+      </x:c>
+      <x:c r="D4" s="46" t="str">
+        <x:v>Grado</x:v>
+      </x:c>
+      <x:c r="E4" s="46" t="str">
+        <x:v>Estilo</x:v>
+      </x:c>
+      <x:c r="F4" s="46" t="str">
+        <x:v>Intentos</x:v>
+      </x:c>
+      <x:c r="G4" s="46" t="str">
+        <x:v>Observaciones</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="53" customHeight="1">
+      <x:c r="A5" s="48" t="d">
+        <x:v>2026-10-14T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B5" s="42" t="str">
+        <x:v>Námaste</x:v>
+      </x:c>
+      <x:c r="C5" s="42" t="str">
+        <x:v>Archidona</x:v>
+      </x:c>
+      <x:c r="D5" s="42" t="str">
+        <x:v>7c</x:v>
+      </x:c>
+      <x:c r="E5" s="42" t="str">
+        <x:v>Redpoint</x:v>
+      </x:c>
+      <x:c r="F5" s="49"/>
+      <x:c r="G5" s="50" t="str">
+        <x:v>Proyecto pendiente encadenado. Salida recta exigente; el límite fue la salida, más que el dinámico.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="53" customHeight="1">
+      <x:c r="A6" s="51" t="d">
+        <x:v>2026-09-23T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B6" s="52" t="str">
+        <x:v>Moya Boom</x:v>
+      </x:c>
+      <x:c r="C6" s="52" t="str">
+        <x:v>Mijas</x:v>
+      </x:c>
+      <x:c r="D6" s="52" t="str">
+        <x:v>7b+</x:v>
+      </x:c>
+      <x:c r="E6" s="52" t="str">
+        <x:v>Segundo intento</x:v>
+      </x:c>
+      <x:c r="F6" s="53" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="G6" s="54" t="str">
+        <x:v>Fecha del registro de 8a.nu. El usuario la recordó aproximadamente como hace dos semanas.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="42"/>
+      <x:c r="B7" s="42"/>
+      <x:c r="C7" s="42"/>
+      <x:c r="D7" s="42"/>
+      <x:c r="E7" s="42"/>
+      <x:c r="F7" s="42"/>
+      <x:c r="G7" s="42"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="55" t="str">
+        <x:v>Fuente: 8a.nu. Perfil consultado el 15/10/2026. Intentos de Námaste no registrados.</x:v>
+      </x:c>
+      <x:c r="B8" s="55"/>
+      <x:c r="C8" s="55"/>
+      <x:c r="D8" s="55"/>
+      <x:c r="E8" s="55"/>
+      <x:c r="F8" s="55"/>
+      <x:c r="G8" s="55"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="55" t="str">
+        <x:v>https://www.8a.nu/user/juanfran-jimenez/sportclimbing</x:v>
+      </x:c>
+      <x:c r="B9" s="55"/>
+      <x:c r="C9" s="55"/>
+      <x:c r="D9" s="55"/>
+      <x:c r="E9" s="55"/>
+      <x:c r="F9" s="55"/>
+      <x:c r="G9" s="55"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="42"/>
+      <x:c r="B10" s="42"/>
+      <x:c r="C10" s="42"/>
+      <x:c r="D10" s="42"/>
+      <x:c r="E10" s="42"/>
+      <x:c r="F10" s="42"/>
+      <x:c r="G10" s="42"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="42"/>
+      <x:c r="B11" s="42"/>
+      <x:c r="C11" s="42"/>
+      <x:c r="D11" s="42"/>
+      <x:c r="E11" s="42"/>
+      <x:c r="F11" s="42"/>
+      <x:c r="G11" s="42"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="56" t="str">
+        <x:v>Test de fuerza con sensor</x:v>
+      </x:c>
+      <x:c r="B12" s="42"/>
+      <x:c r="C12" s="42"/>
+      <x:c r="D12" s="42"/>
+      <x:c r="E12" s="42"/>
+      <x:c r="F12" s="42"/>
+      <x:c r="G12" s="42"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="42"/>
+      <x:c r="B13" s="42"/>
+      <x:c r="C13" s="42"/>
+      <x:c r="D13" s="42"/>
+      <x:c r="E13" s="42"/>
+      <x:c r="F13" s="42"/>
+      <x:c r="G13" s="42"/>
+    </x:row>
+    <x:row r="14" ht="27" customHeight="1">
+      <x:c r="A14" s="46" t="str">
+        <x:v>Actualizado</x:v>
+      </x:c>
+      <x:c r="B14" s="46" t="str">
+        <x:v>Estado</x:v>
+      </x:c>
+      <x:c r="C14" s="46" t="str">
+        <x:v>Resultado</x:v>
+      </x:c>
+      <x:c r="D14" s="42"/>
+      <x:c r="E14" s="42"/>
+      <x:c r="F14" s="42"/>
+      <x:c r="G14" s="42"/>
+    </x:row>
+    <x:row r="15" ht="25" customHeight="1">
+      <x:c r="A15" s="48" t="d">
+        <x:v>2026-10-15T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B15" s="42" t="str">
+        <x:v>Pendiente</x:v>
+      </x:c>
+      <x:c r="C15" s="42" t="str">
+        <x:v>Sin medición</x:v>
+      </x:c>
+      <x:c r="D15" s="42"/>
+      <x:c r="E15" s="42"/>
+      <x:c r="F15" s="42"/>
+      <x:c r="G15" s="42"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="42"/>
+      <x:c r="B16" s="42"/>
+      <x:c r="C16" s="42"/>
+      <x:c r="D16" s="42"/>
+      <x:c r="E16" s="42"/>
+      <x:c r="F16" s="42"/>
+      <x:c r="G16" s="42"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="55" t="str">
+        <x:v>Fuente: confirmación del usuario el 15/10/2026.</x:v>
+      </x:c>
+      <x:c r="B17" s="42"/>
+      <x:c r="C17" s="42"/>
+      <x:c r="D17" s="42"/>
+      <x:c r="E17" s="42"/>
+      <x:c r="F17" s="42"/>
+      <x:c r="G17" s="42"/>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Rediseña cuaderno de entrenamiento con calendario y Logbook actualizado
</commit_message>
<xml_diff>
--- a/escalada/moonboard_entrenamientos.xlsx
+++ b/escalada/moonboard_entrenamientos.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sesiones MoonBoard" sheetId="1" r:id="R539f280df7354f30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuerda y sensor" sheetId="2" r:id="R0a7f6f0e316c4656"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sesiones MoonBoard" sheetId="1" r:id="Rc73a28d4ec4641b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuerda y sensor" sheetId="2" r:id="Re2ea6f6e0d6348f5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -301,8 +301,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MoonBoardSessions" displayName="MoonBoardSessions" ref="A11:H20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A11:H20"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MoonBoardSessions" displayName="MoonBoardSessions" ref="A11:H27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A11:H27"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Fecha"/>
     <x:tableColumn id="2" name="Problemas"/>
@@ -542,7 +542,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>Sesiones registradas entre el 17 de agosto y el 17 de septiembre de 2026</x:v>
+        <x:v>Sesiones registradas entre el 17 de agosto y el 13 de octubre de 2026</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -572,29 +572,29 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="n">
-        <x:f>COUNTA(A12:A20)</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTA(A12:A27)</x:f>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B6" s="5"/>
       <x:c r="C6" s="5" t="n">
-        <x:f>SUM(B12:B20)</x:f>
-        <x:v>141</x:v>
+        <x:f>SUM(B12:B27)</x:f>
+        <x:v>261</x:v>
       </x:c>
       <x:c r="D6" s="5"/>
       <x:c r="E6" s="5" t="n">
-        <x:f>SUM(C12:C20)</x:f>
-        <x:v>108</x:v>
+        <x:f>SUM(C12:C27)</x:f>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="8" t="n">
-        <x:f>SUM(C12:C20)/SUM(B12:B20)</x:f>
-        <x:v>0.7659574468085106</x:v>
+        <x:f>SUM(C12:C27)/SUM(B12:B27)</x:f>
+        <x:v>0.7509578544061303</x:v>
       </x:c>
       <x:c r="H6" s="5"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="9" t="str">
-        <x:v>Fuente: registro Logbook de la app MoonBoard en Android, consultado el 17/09/2026.</x:v>
+        <x:v>Fuente: Logbook de MoonBoard en Android, consultado por USB el 15/10/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -624,59 +624,59 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
-      <x:c r="A12" s="30" t="n">
-        <x:v>46282</x:v>
+      <x:c r="A12" s="30" t="d">
+        <x:v>2026-10-13T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B12" s="31" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="C12" s="31" t="n">
-        <x:v>14</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D12" s="31" t="n">
         <x:f>B12-C12</x:f>
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E12" s="31" t="n">
-        <x:v>25</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F12" s="32" t="n">
         <x:f>C12/B12</x:f>
-        <x:v>0.7</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="G12" s="33" t="n">
         <x:f>E12/B12</x:f>
-        <x:v>1.25</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="H12" s="34" t="n">
         <x:f>A12-A13</x:f>
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
-      <x:c r="A13" s="30" t="n">
-        <x:v>46280</x:v>
+      <x:c r="A13" s="30" t="d">
+        <x:v>2026-10-06T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B13" s="31" t="n">
-        <x:v>16</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C13" s="31" t="n">
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D13" s="31" t="n">
         <x:f>B13-C13</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E13" s="31" t="n">
-        <x:v>25</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F13" s="32" t="n">
         <x:f>C13/B13</x:f>
-        <x:v>0.6875</x:v>
+        <x:v>0.6153846153846154</x:v>
       </x:c>
       <x:c r="G13" s="33" t="n">
         <x:f>E13/B13</x:f>
-        <x:v>1.5625</x:v>
+        <x:v>1.5384615384615385</x:v>
       </x:c>
       <x:c r="H13" s="34" t="n">
         <x:f>A13-A14</x:f>
@@ -684,149 +684,149 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
-      <x:c r="A14" s="30" t="n">
-        <x:v>46275</x:v>
+      <x:c r="A14" s="30" t="d">
+        <x:v>2026-10-01T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B14" s="31" t="n">
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C14" s="31" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D14" s="31" t="n">
         <x:f>B14-C14</x:f>
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E14" s="31" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F14" s="32" t="n">
         <x:f>C14/B14</x:f>
-        <x:v>0.6153846153846154</x:v>
+        <x:v>0.5625</x:v>
       </x:c>
       <x:c r="G14" s="33" t="n">
         <x:f>E14/B14</x:f>
-        <x:v>1.5384615384615385</x:v>
+        <x:v>1.375</x:v>
       </x:c>
       <x:c r="H14" s="34" t="n">
         <x:f>A14-A15</x:f>
-        <x:v>7</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
-      <x:c r="A15" s="30" t="n">
-        <x:v>46268</x:v>
+      <x:c r="A15" s="30" t="d">
+        <x:v>2026-09-29T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B15" s="31" t="n">
-        <x:v>17</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C15" s="31" t="n">
-        <x:v>15</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D15" s="31" t="n">
         <x:f>B15-C15</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E15" s="31" t="n">
-        <x:v>23</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F15" s="32" t="n">
         <x:f>C15/B15</x:f>
-        <x:v>0.8823529411764706</x:v>
+        <x:v>0.8620689655172413</x:v>
       </x:c>
       <x:c r="G15" s="33" t="n">
         <x:f>E15/B15</x:f>
-        <x:v>1.3529411764705883</x:v>
+        <x:v>1.3103448275862069</x:v>
       </x:c>
       <x:c r="H15" s="34" t="n">
         <x:f>A15-A16</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
-      <x:c r="A16" s="30" t="n">
-        <x:v>46266</x:v>
+      <x:c r="A16" s="30" t="d">
+        <x:v>2026-09-24T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B16" s="31" t="n">
-        <x:v>15</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C16" s="31" t="n">
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D16" s="31" t="n">
         <x:f>B16-C16</x:f>
-        <x:v>4</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E16" s="31" t="n">
-        <x:v>21</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F16" s="32" t="n">
         <x:f>C16/B16</x:f>
-        <x:v>0.7333333333333333</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G16" s="33" t="n">
         <x:f>E16/B16</x:f>
-        <x:v>1.4</x:v>
+        <x:v>1.625</x:v>
       </x:c>
       <x:c r="H16" s="34" t="n">
         <x:f>A16-A17</x:f>
-        <x:v>5</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
-      <x:c r="A17" s="30" t="n">
-        <x:v>46261</x:v>
+      <x:c r="A17" s="30" t="d">
+        <x:v>2026-09-21T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B17" s="31" t="n">
         <x:v>18</x:v>
       </x:c>
       <x:c r="C17" s="31" t="n">
-        <x:v>16</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D17" s="31" t="n">
         <x:f>B17-C17</x:f>
-        <x:v>2</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E17" s="31" t="n">
-        <x:v>22</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F17" s="32" t="n">
         <x:f>C17/B17</x:f>
-        <x:v>0.8888888888888888</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="G17" s="33" t="n">
         <x:f>E17/B17</x:f>
-        <x:v>1.2222222222222223</x:v>
+        <x:v>1.4444444444444444</x:v>
       </x:c>
       <x:c r="H17" s="34" t="n">
         <x:f>A17-A18</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
-      <x:c r="A18" s="30" t="n">
-        <x:v>46256</x:v>
+      <x:c r="A18" s="30" t="d">
+        <x:v>2026-09-19T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B18" s="31" t="n">
-        <x:v>11</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="31" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D18" s="31" t="n">
         <x:f>B18-C18</x:f>
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E18" s="31" t="n">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F18" s="32" t="n">
         <x:f>C18/B18</x:f>
-        <x:v>0.5454545454545454</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="G18" s="33" t="n">
         <x:f>E18/B18</x:f>
-        <x:v>1.8181818181818181</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="H18" s="34" t="n">
         <x:f>A18-A19</x:f>
@@ -834,64 +834,274 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
-      <x:c r="A19" s="30" t="n">
-        <x:v>46254</x:v>
+      <x:c r="A19" s="30" t="d">
+        <x:v>2026-09-17T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B19" s="31" t="n">
-        <x:v>17</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C19" s="31" t="n">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D19" s="31" t="n">
         <x:f>B19-C19</x:f>
-        <x:v>4</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="31" t="n">
-        <x:v>20</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F19" s="32" t="n">
         <x:f>C19/B19</x:f>
-        <x:v>0.7647058823529411</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="G19" s="33" t="n">
         <x:f>E19/B19</x:f>
-        <x:v>1.1764705882352942</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="H19" s="34" t="n">
         <x:f>A19-A20</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
-      <x:c r="A20" s="35" t="n">
-        <x:v>46251</x:v>
+      <x:c r="A20" s="35" t="d">
+        <x:v>2026-09-15T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B20" s="36" t="n">
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C20" s="36" t="n">
-        <x:v>14</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D20" s="36" t="n">
         <x:f>B20-C20</x:f>
-        <x:v>0</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E20" s="36" t="n">
-        <x:v>15</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F20" s="37" t="n">
         <x:f>C20/B20</x:f>
-        <x:v>1</x:v>
+        <x:v>0.6875</x:v>
       </x:c>
       <x:c r="G20" s="38" t="n">
         <x:f>E20/B20</x:f>
+        <x:v>1.5625</x:v>
+      </x:c>
+      <x:c r="H20" s="39" t="n">
+        <x:f>A20-A21</x:f>
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="30" t="d">
+        <x:v>2026-09-10T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B21" s="31" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="C21" s="31" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="D21" s="31" t="n">
+        <x:f>B21-C21</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E21" s="31" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F21" s="32" t="n">
+        <x:f>C21/B21</x:f>
+        <x:v>0.6153846153846154</x:v>
+      </x:c>
+      <x:c r="G21" s="33" t="n">
+        <x:f>E21/B21</x:f>
+        <x:v>1.5384615384615385</x:v>
+      </x:c>
+      <x:c r="H21" s="34" t="n">
+        <x:f>A21-A22</x:f>
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="30" t="d">
+        <x:v>2026-09-03T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B22" s="31" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C22" s="31" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="D22" s="31" t="n">
+        <x:f>B22-C22</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E22" s="31" t="n">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F22" s="32" t="n">
+        <x:f>C22/B22</x:f>
+        <x:v>0.8823529411764706</x:v>
+      </x:c>
+      <x:c r="G22" s="33" t="n">
+        <x:f>E22/B22</x:f>
+        <x:v>1.3529411764705883</x:v>
+      </x:c>
+      <x:c r="H22" s="34" t="n">
+        <x:f>A22-A23</x:f>
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="30" t="d">
+        <x:v>2026-09-01T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B23" s="31" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="C23" s="31" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="D23" s="31" t="n">
+        <x:f>B23-C23</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E23" s="31" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F23" s="32" t="n">
+        <x:f>C23/B23</x:f>
+        <x:v>0.7333333333333333</x:v>
+      </x:c>
+      <x:c r="G23" s="33" t="n">
+        <x:f>E23/B23</x:f>
+        <x:v>1.4</x:v>
+      </x:c>
+      <x:c r="H23" s="34" t="n">
+        <x:f>A23-A24</x:f>
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="30" t="d">
+        <x:v>2026-08-27T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B24" s="31" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="C24" s="31" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="D24" s="31" t="n">
+        <x:f>B24-C24</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E24" s="31" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F24" s="32" t="n">
+        <x:f>C24/B24</x:f>
+        <x:v>0.8888888888888888</x:v>
+      </x:c>
+      <x:c r="G24" s="33" t="n">
+        <x:f>E24/B24</x:f>
+        <x:v>1.2222222222222223</x:v>
+      </x:c>
+      <x:c r="H24" s="34" t="n">
+        <x:f>A24-A25</x:f>
+        <x:v>5</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="30" t="d">
+        <x:v>2026-08-22T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B25" s="31" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C25" s="31" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D25" s="31" t="n">
+        <x:f>B25-C25</x:f>
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E25" s="31" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F25" s="32" t="n">
+        <x:f>C25/B25</x:f>
+        <x:v>0.5454545454545454</x:v>
+      </x:c>
+      <x:c r="G25" s="33" t="n">
+        <x:f>E25/B25</x:f>
+        <x:v>1.8181818181818181</x:v>
+      </x:c>
+      <x:c r="H25" s="34" t="n">
+        <x:f>A25-A26</x:f>
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="30" t="d">
+        <x:v>2026-08-20T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B26" s="31" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C26" s="31" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="D26" s="31" t="n">
+        <x:f>B26-C26</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E26" s="31" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F26" s="32" t="n">
+        <x:f>C26/B26</x:f>
+        <x:v>0.7647058823529411</x:v>
+      </x:c>
+      <x:c r="G26" s="33" t="n">
+        <x:f>E26/B26</x:f>
+        <x:v>1.1764705882352942</x:v>
+      </x:c>
+      <x:c r="H26" s="34" t="n">
+        <x:f>A26-A27</x:f>
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="30" t="d">
+        <x:v>2026-08-17T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B27" s="31" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C27" s="31" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D27" s="31" t="n">
+        <x:f>B27-C27</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E27" s="31" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F27" s="32" t="n">
+        <x:f>C27/B27</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G27" s="33" t="n">
+        <x:f>E27/B27</x:f>
         <x:v>1.0714285714285714</x:v>
       </x:c>
-      <x:c r="H20" s="39"/>
+      <x:c r="H27" s="34"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F12:F20">
+  <x:conditionalFormatting sqref="F12:F27">
     <x:cfRule type="colorScale" priority="1">
       <x:colorScale>
         <x:cfvo type="min"/>
@@ -905,7 +1115,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70b3b0de441e4259"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09277f980e4845db"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Importa la sesión de fuerza del 16 de octubre y revisa el bloque 2
</commit_message>
<xml_diff>
--- a/escalada/moonboard_entrenamientos.xlsx
+++ b/escalada/moonboard_entrenamientos.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sesiones MoonBoard" sheetId="1" r:id="Rc73a28d4ec4641b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuerda y sensor" sheetId="2" r:id="Re2ea6f6e0d6348f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sesiones MoonBoard" sheetId="1" r:id="R8fe53255dcc64c81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuerda y sensor" sheetId="2" r:id="Rd94926f9091648d7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -301,8 +301,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MoonBoardSessions" displayName="MoonBoardSessions" ref="A11:H27" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A11:H27"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="MoonBoardSessions" displayName="MoonBoardSessions" ref="A11:H28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A11:H28"/>
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Fecha"/>
     <x:tableColumn id="2" name="Problemas"/>
@@ -542,7 +542,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>Sesiones registradas entre el 17 de agosto y el 13 de octubre de 2026</x:v>
+        <x:v>Sesiones registradas entre el 17 de agosto y el 16 de octubre de 2026</x:v>
       </x:c>
       <x:c r="B3" s="4"/>
       <x:c r="C3" s="4"/>
@@ -572,29 +572,29 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="7" t="n">
-        <x:f>COUNTA(A12:A27)</x:f>
-        <x:v>16</x:v>
+        <x:f>COUNTA(A12:A28)</x:f>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B6" s="5"/>
       <x:c r="C6" s="5" t="n">
-        <x:f>SUM(B12:B27)</x:f>
-        <x:v>261</x:v>
+        <x:f>SUM(B12:B28)</x:f>
+        <x:v>278</x:v>
       </x:c>
       <x:c r="D6" s="5"/>
       <x:c r="E6" s="5" t="n">
-        <x:f>SUM(C12:C27)</x:f>
-        <x:v>196</x:v>
+        <x:f>SUM(C12:C28)</x:f>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="F6" s="5"/>
       <x:c r="G6" s="8" t="n">
-        <x:f>SUM(C12:C27)/SUM(B12:B27)</x:f>
-        <x:v>0.7509578544061303</x:v>
+        <x:f>SUM(C12:C28)/SUM(B12:B28)</x:f>
+        <x:v>0.7446043165467626</x:v>
       </x:c>
       <x:c r="H6" s="5"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="9" t="str">
-        <x:v>Fuente: Logbook de MoonBoard en Android, consultado por USB el 15/10/2026.</x:v>
+        <x:v>Fuente: Logbook de MoonBoard en Android, consultado por USB el 16/10/2026.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="30" customHeight="1">
@@ -625,208 +625,208 @@
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="30" t="d">
-        <x:v>2026-10-13T12:00:00.000Z</x:v>
+        <x:v>2026-10-16T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B12" s="31" t="n">
-        <x:v>20</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C12" s="31" t="n">
-        <x:v>19</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D12" s="31" t="n">
         <x:f>B12-C12</x:f>
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E12" s="31" t="n">
-        <x:v>22</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F12" s="32" t="n">
         <x:f>C12/B12</x:f>
-        <x:v>0.95</x:v>
+        <x:v>0.6470588235294118</x:v>
       </x:c>
       <x:c r="G12" s="33" t="n">
         <x:f>E12/B12</x:f>
-        <x:v>1.1</x:v>
+        <x:v>1.5294117647058822</x:v>
       </x:c>
       <x:c r="H12" s="34" t="n">
         <x:f>A12-A13</x:f>
-        <x:v>7</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="30" t="d">
-        <x:v>2026-10-06T12:00:00.000Z</x:v>
+        <x:v>2026-10-13T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B13" s="31" t="n">
-        <x:v>13</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C13" s="31" t="n">
-        <x:v>8</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D13" s="31" t="n">
         <x:f>B13-C13</x:f>
-        <x:v>5</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E13" s="31" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F13" s="32" t="n">
         <x:f>C13/B13</x:f>
-        <x:v>0.6153846153846154</x:v>
+        <x:v>0.95</x:v>
       </x:c>
       <x:c r="G13" s="33" t="n">
         <x:f>E13/B13</x:f>
-        <x:v>1.5384615384615385</x:v>
+        <x:v>1.1</x:v>
       </x:c>
       <x:c r="H13" s="34" t="n">
         <x:f>A13-A14</x:f>
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="30" t="d">
-        <x:v>2026-10-01T12:00:00.000Z</x:v>
+        <x:v>2026-10-06T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B14" s="31" t="n">
-        <x:v>16</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C14" s="31" t="n">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D14" s="31" t="n">
         <x:f>B14-C14</x:f>
-        <x:v>7</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E14" s="31" t="n">
-        <x:v>22</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F14" s="32" t="n">
         <x:f>C14/B14</x:f>
-        <x:v>0.5625</x:v>
+        <x:v>0.6153846153846154</x:v>
       </x:c>
       <x:c r="G14" s="33" t="n">
         <x:f>E14/B14</x:f>
-        <x:v>1.375</x:v>
+        <x:v>1.5384615384615385</x:v>
       </x:c>
       <x:c r="H14" s="34" t="n">
         <x:f>A14-A15</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="30" t="d">
-        <x:v>2026-09-29T12:00:00.000Z</x:v>
+        <x:v>2026-10-01T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B15" s="31" t="n">
-        <x:v>29</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C15" s="31" t="n">
-        <x:v>25</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="D15" s="31" t="n">
         <x:f>B15-C15</x:f>
-        <x:v>4</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E15" s="31" t="n">
-        <x:v>38</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F15" s="32" t="n">
         <x:f>C15/B15</x:f>
-        <x:v>0.8620689655172413</x:v>
+        <x:v>0.5625</x:v>
       </x:c>
       <x:c r="G15" s="33" t="n">
         <x:f>E15/B15</x:f>
-        <x:v>1.3103448275862069</x:v>
+        <x:v>1.375</x:v>
       </x:c>
       <x:c r="H15" s="34" t="n">
         <x:f>A15-A16</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="30" t="d">
-        <x:v>2026-09-24T12:00:00.000Z</x:v>
+        <x:v>2026-09-29T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B16" s="31" t="n">
-        <x:v>16</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C16" s="31" t="n">
-        <x:v>8</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D16" s="31" t="n">
         <x:f>B16-C16</x:f>
-        <x:v>8</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E16" s="31" t="n">
-        <x:v>26</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="F16" s="32" t="n">
         <x:f>C16/B16</x:f>
-        <x:v>0.5</x:v>
+        <x:v>0.8620689655172413</x:v>
       </x:c>
       <x:c r="G16" s="33" t="n">
         <x:f>E16/B16</x:f>
-        <x:v>1.625</x:v>
+        <x:v>1.3103448275862069</x:v>
       </x:c>
       <x:c r="H16" s="34" t="n">
         <x:f>A16-A17</x:f>
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="30" t="d">
-        <x:v>2026-09-21T12:00:00.000Z</x:v>
+        <x:v>2026-09-24T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B17" s="31" t="n">
-        <x:v>18</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C17" s="31" t="n">
-        <x:v>12</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D17" s="31" t="n">
         <x:f>B17-C17</x:f>
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E17" s="31" t="n">
         <x:v>26</x:v>
       </x:c>
       <x:c r="F17" s="32" t="n">
         <x:f>C17/B17</x:f>
-        <x:v>0.6666666666666666</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="G17" s="33" t="n">
         <x:f>E17/B17</x:f>
-        <x:v>1.4444444444444444</x:v>
+        <x:v>1.625</x:v>
       </x:c>
       <x:c r="H17" s="34" t="n">
         <x:f>A17-A18</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="30" t="d">
-        <x:v>2026-09-19T12:00:00.000Z</x:v>
+        <x:v>2026-09-21T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B18" s="31" t="n">
-        <x:v>8</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C18" s="31" t="n">
-        <x:v>7</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D18" s="31" t="n">
         <x:f>B18-C18</x:f>
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E18" s="31" t="n">
-        <x:v>10</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="F18" s="32" t="n">
         <x:f>C18/B18</x:f>
-        <x:v>0.875</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="G18" s="33" t="n">
         <x:f>E18/B18</x:f>
-        <x:v>1.25</x:v>
+        <x:v>1.4444444444444444</x:v>
       </x:c>
       <x:c r="H18" s="34" t="n">
         <x:f>A18-A19</x:f>
@@ -835,24 +835,24 @@
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="30" t="d">
-        <x:v>2026-09-17T12:00:00.000Z</x:v>
+        <x:v>2026-09-19T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B19" s="31" t="n">
-        <x:v>20</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="31" t="n">
-        <x:v>14</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D19" s="31" t="n">
         <x:f>B19-C19</x:f>
-        <x:v>6</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="E19" s="31" t="n">
-        <x:v>25</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F19" s="32" t="n">
         <x:f>C19/B19</x:f>
-        <x:v>0.7</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="G19" s="33" t="n">
         <x:f>E19/B19</x:f>
@@ -865,148 +865,148 @@
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="35" t="d">
-        <x:v>2026-09-15T12:00:00.000Z</x:v>
+        <x:v>2026-09-17T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B20" s="36" t="n">
-        <x:v>16</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C20" s="36" t="n">
-        <x:v>11</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="D20" s="36" t="n">
         <x:f>B20-C20</x:f>
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="36" t="n">
         <x:v>25</x:v>
       </x:c>
       <x:c r="F20" s="37" t="n">
         <x:f>C20/B20</x:f>
-        <x:v>0.6875</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="G20" s="38" t="n">
         <x:f>E20/B20</x:f>
-        <x:v>1.5625</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="H20" s="39" t="n">
         <x:f>A20-A21</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="30" t="d">
-        <x:v>2026-09-10T12:00:00.000Z</x:v>
+        <x:v>2026-09-15T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B21" s="31" t="n">
-        <x:v>13</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C21" s="31" t="n">
-        <x:v>8</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D21" s="31" t="n">
         <x:f>B21-C21</x:f>
         <x:v>5</x:v>
       </x:c>
       <x:c r="E21" s="31" t="n">
-        <x:v>20</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F21" s="32" t="n">
         <x:f>C21/B21</x:f>
-        <x:v>0.6153846153846154</x:v>
+        <x:v>0.6875</x:v>
       </x:c>
       <x:c r="G21" s="33" t="n">
         <x:f>E21/B21</x:f>
-        <x:v>1.5384615384615385</x:v>
+        <x:v>1.5625</x:v>
       </x:c>
       <x:c r="H21" s="34" t="n">
         <x:f>A21-A22</x:f>
-        <x:v>7</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="30" t="d">
-        <x:v>2026-09-03T12:00:00.000Z</x:v>
+        <x:v>2026-09-10T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B22" s="31" t="n">
-        <x:v>17</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C22" s="31" t="n">
-        <x:v>15</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D22" s="31" t="n">
         <x:f>B22-C22</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E22" s="31" t="n">
-        <x:v>23</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F22" s="32" t="n">
         <x:f>C22/B22</x:f>
-        <x:v>0.8823529411764706</x:v>
+        <x:v>0.6153846153846154</x:v>
       </x:c>
       <x:c r="G22" s="33" t="n">
         <x:f>E22/B22</x:f>
-        <x:v>1.3529411764705883</x:v>
+        <x:v>1.5384615384615385</x:v>
       </x:c>
       <x:c r="H22" s="34" t="n">
         <x:f>A22-A23</x:f>
-        <x:v>2</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="30" t="d">
-        <x:v>2026-09-01T12:00:00.000Z</x:v>
+        <x:v>2026-09-03T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B23" s="31" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="C23" s="31" t="n">
         <x:v>15</x:v>
-      </x:c>
-      <x:c r="C23" s="31" t="n">
-        <x:v>11</x:v>
       </x:c>
       <x:c r="D23" s="31" t="n">
         <x:f>B23-C23</x:f>
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E23" s="31" t="n">
-        <x:v>21</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F23" s="32" t="n">
         <x:f>C23/B23</x:f>
-        <x:v>0.7333333333333333</x:v>
+        <x:v>0.8823529411764706</x:v>
       </x:c>
       <x:c r="G23" s="33" t="n">
         <x:f>E23/B23</x:f>
-        <x:v>1.4</x:v>
+        <x:v>1.3529411764705883</x:v>
       </x:c>
       <x:c r="H23" s="34" t="n">
         <x:f>A23-A24</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="30" t="d">
-        <x:v>2026-08-27T12:00:00.000Z</x:v>
+        <x:v>2026-09-01T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B24" s="31" t="n">
-        <x:v>18</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C24" s="31" t="n">
-        <x:v>16</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D24" s="31" t="n">
         <x:f>B24-C24</x:f>
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E24" s="31" t="n">
-        <x:v>22</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="F24" s="32" t="n">
         <x:f>C24/B24</x:f>
-        <x:v>0.8888888888888888</x:v>
+        <x:v>0.7333333333333333</x:v>
       </x:c>
       <x:c r="G24" s="33" t="n">
         <x:f>E24/B24</x:f>
-        <x:v>1.2222222222222223</x:v>
+        <x:v>1.4</x:v>
       </x:c>
       <x:c r="H24" s="34" t="n">
         <x:f>A24-A25</x:f>
@@ -1015,93 +1015,123 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="30" t="d">
-        <x:v>2026-08-22T12:00:00.000Z</x:v>
+        <x:v>2026-08-27T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B25" s="31" t="n">
-        <x:v>11</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C25" s="31" t="n">
-        <x:v>6</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="D25" s="31" t="n">
         <x:f>B25-C25</x:f>
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E25" s="31" t="n">
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="F25" s="32" t="n">
         <x:f>C25/B25</x:f>
-        <x:v>0.5454545454545454</x:v>
+        <x:v>0.8888888888888888</x:v>
       </x:c>
       <x:c r="G25" s="33" t="n">
         <x:f>E25/B25</x:f>
-        <x:v>1.8181818181818181</x:v>
+        <x:v>1.2222222222222223</x:v>
       </x:c>
       <x:c r="H25" s="34" t="n">
         <x:f>A25-A26</x:f>
-        <x:v>2</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="30" t="d">
-        <x:v>2026-08-20T12:00:00.000Z</x:v>
+        <x:v>2026-08-22T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B26" s="31" t="n">
-        <x:v>17</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C26" s="31" t="n">
-        <x:v>13</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D26" s="31" t="n">
         <x:f>B26-C26</x:f>
-        <x:v>4</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="E26" s="31" t="n">
         <x:v>20</x:v>
       </x:c>
       <x:c r="F26" s="32" t="n">
         <x:f>C26/B26</x:f>
-        <x:v>0.7647058823529411</x:v>
+        <x:v>0.5454545454545454</x:v>
       </x:c>
       <x:c r="G26" s="33" t="n">
         <x:f>E26/B26</x:f>
-        <x:v>1.1764705882352942</x:v>
+        <x:v>1.8181818181818181</x:v>
       </x:c>
       <x:c r="H26" s="34" t="n">
         <x:f>A26-A27</x:f>
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="30" t="d">
-        <x:v>2026-08-17T12:00:00.000Z</x:v>
+        <x:v>2026-08-20T12:00:00.000Z</x:v>
       </x:c>
       <x:c r="B27" s="31" t="n">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C27" s="31" t="n">
-        <x:v>14</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D27" s="31" t="n">
         <x:f>B27-C27</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E27" s="31" t="n">
-        <x:v>15</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F27" s="32" t="n">
         <x:f>C27/B27</x:f>
-        <x:v>1</x:v>
+        <x:v>0.7647058823529411</x:v>
       </x:c>
       <x:c r="G27" s="33" t="n">
         <x:f>E27/B27</x:f>
+        <x:v>1.1764705882352942</x:v>
+      </x:c>
+      <x:c r="H27" s="34" t="n">
+        <x:f>A27-A28</x:f>
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="30" t="d">
+        <x:v>2026-08-17T12:00:00.000Z</x:v>
+      </x:c>
+      <x:c r="B28" s="31" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C28" s="31" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D28" s="31" t="n">
+        <x:f>B28-C28</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E28" s="31" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F28" s="32" t="n">
+        <x:f>C28/B28</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G28" s="33" t="n">
+        <x:f>E28/B28</x:f>
         <x:v>1.0714285714285714</x:v>
       </x:c>
-      <x:c r="H27" s="34"/>
+      <x:c r="H28" s="34"/>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="F12:F27">
+  <x:conditionalFormatting sqref="F12:F28">
     <x:cfRule type="colorScale" priority="1">
       <x:colorScale>
         <x:cfvo type="min"/>
@@ -1115,7 +1145,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R09277f980e4845db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ed45fdb5a1b4b1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>